<commit_message>
Replace unverifiable formula in keyword plan workbook
LibreOffice is unavailable in this environment - it times out on even a
three-cell file - so formulas cannot be recalculated and verified here.

Removed the _xlfn.MINIFS Best Position formula, which carries the most
compatibility risk and could not be checked. That column is now a
static snapshot of current Semrush rankings, labelled as such.

The remaining COUNTIF, COUNTIFS and SUMIF formulas on Page Summary are
Excel-2007-era and universally supported; their expected output was
verified independently in Python against the same source data. They
populate when Excel opens the file. The README notes this.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AT1mcba4Jj4VCrR3QX7ZKS
</commit_message>
<xml_diff>
--- a/betterwaste-kw-audit/Better_Waste_Keyword_Plan.xlsx
+++ b/betterwaste-kw-audit/Better_Waste_Keyword_Plan.xlsx
@@ -578,7 +578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -832,13 +832,25 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="28" customHeight="1">
+    <row r="27" ht="42" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
+          <t>Formulas</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>The Keywords, Total SV and Already Ranking columns on Page Summary are live COUNTIF/SUMIF formulas. They show no value until Excel opens and recalculates the file — that is expected. Best Position is a static snapshot of current Semrush rankings, not a formula.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
           <t>Not verified</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>The Manchester / London / Birmingham city URLs return 301 while the "-old" equivalents return 200. Confirm where those redirects point before acting — see the Fix List.</t>
         </is>
@@ -11902,7 +11914,7 @@
       </c>
       <c r="H1" s="5" t="inlineStr">
         <is>
-          <t>Best Position</t>
+          <t>Best Position (snapshot)</t>
         </is>
       </c>
     </row>
@@ -11939,9 +11951,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A2,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H2" s="14">
-        <f>IF(G2=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A2,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H2" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -11977,9 +11990,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A3,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H3" s="14">
-        <f>IF(G3=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A3,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H3" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -12015,9 +12029,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A4,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H4" s="14">
-        <f>IF(G4=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A4,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -12053,9 +12068,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A5,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H5" s="14">
-        <f>IF(G5=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A5,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -12091,9 +12107,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A6,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H6" s="14">
-        <f>IF(G6=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A6,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -12129,9 +12146,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A7,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H7" s="14">
-        <f>IF(G7=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A7,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -12167,9 +12185,8 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A8,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H8" s="14">
-        <f>IF(G8=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A8,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H8" s="14" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="9">
@@ -12205,9 +12222,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A9,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H9" s="14">
-        <f>IF(G9=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A9,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -12243,9 +12261,8 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A10,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H10" s="14">
-        <f>IF(G10=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A10,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H10" s="14" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="11">
@@ -12281,9 +12298,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A11,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H11" s="14">
-        <f>IF(G11=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A11,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H11" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -12319,9 +12337,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A12,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H12" s="14">
-        <f>IF(G12=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A12,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -12357,9 +12376,8 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A13,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H13" s="14">
-        <f>IF(G13=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A13,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H13" s="14" t="n">
+        <v>42</v>
       </c>
     </row>
     <row r="14">
@@ -12395,9 +12413,8 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A14,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H14" s="14">
-        <f>IF(G14=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A14,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H14" s="14" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="15">
@@ -12433,9 +12450,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A15,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H15" s="14">
-        <f>IF(G15=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A15,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H15" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -12471,9 +12489,8 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A16,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H16" s="14">
-        <f>IF(G16=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A16,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H16" s="14" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="17">
@@ -12509,9 +12526,8 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A17,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H17" s="14">
-        <f>IF(G17=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A17,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H17" s="14" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="18">
@@ -12547,9 +12563,8 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A18,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H18" s="14">
-        <f>IF(G18=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A18,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H18" s="14" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="19">
@@ -12585,9 +12600,8 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A19,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H19" s="14">
-        <f>IF(G19=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A19,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H19" s="14" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="20">
@@ -12623,9 +12637,8 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A20,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H20" s="14">
-        <f>IF(G20=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A20,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H20" s="14" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="21">
@@ -12661,9 +12674,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A21,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H21" s="14">
-        <f>IF(G21=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A21,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H21" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -12699,9 +12713,8 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A22,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H22" s="14">
-        <f>IF(G22=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A22,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H22" s="14" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="23">
@@ -12737,9 +12750,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A23,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H23" s="14">
-        <f>IF(G23=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A23,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H23" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -12775,9 +12789,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A24,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H24" s="14">
-        <f>IF(G24=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A24,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H24" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -12813,9 +12828,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A25,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H25" s="14">
-        <f>IF(G25=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A25,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H25" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -12851,9 +12867,8 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A26,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H26" s="14">
-        <f>IF(G26=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A26,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H26" s="14" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="27">
@@ -12889,9 +12904,8 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A27,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H27" s="14">
-        <f>IF(G27=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A27,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H27" s="14" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="28">
@@ -12927,9 +12941,8 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A28,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H28" s="14">
-        <f>IF(G28=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A28,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H28" s="14" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="29">
@@ -12965,9 +12978,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A29,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H29" s="14">
-        <f>IF(G29=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A29,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H29" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -13003,9 +13017,8 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A30,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H30" s="14">
-        <f>IF(G30=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A30,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H30" s="14" t="n">
+        <v>39</v>
       </c>
     </row>
     <row r="31">
@@ -13041,9 +13054,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A31,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H31" s="14">
-        <f>IF(G31=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A31,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H31" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -13079,9 +13093,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A32,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H32" s="14">
-        <f>IF(G32=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A32,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H32" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -13117,9 +13132,8 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A33,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H33" s="14">
-        <f>IF(G33=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A33,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H33" s="14" t="n">
+        <v>54</v>
       </c>
     </row>
     <row r="34">
@@ -13155,9 +13169,8 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A34,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H34" s="14">
-        <f>IF(G34=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A34,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H34" s="14" t="n">
+        <v>54</v>
       </c>
     </row>
     <row r="35">
@@ -13193,9 +13206,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A35,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H35" s="14">
-        <f>IF(G35=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A35,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H35" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -13231,9 +13245,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A36,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H36" s="14">
-        <f>IF(G36=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A36,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H36" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -13269,9 +13284,8 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A37,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H37" s="14">
-        <f>IF(G37=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A37,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H37" s="14" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="38">
@@ -13307,9 +13321,8 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A38,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H38" s="14">
-        <f>IF(G38=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A38,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H38" s="14" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="39">
@@ -13345,9 +13358,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A39,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H39" s="14">
-        <f>IF(G39=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A39,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H39" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -13383,9 +13397,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A40,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H40" s="14">
-        <f>IF(G40=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A40,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H40" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -13421,9 +13436,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A41,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H41" s="14">
-        <f>IF(G41=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A41,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H41" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="42">
@@ -13459,9 +13475,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A42,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H42" s="14">
-        <f>IF(G42=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A42,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H42" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -13497,9 +13514,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A43,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H43" s="14">
-        <f>IF(G43=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A43,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H43" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -13535,9 +13553,8 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A44,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H44" s="14">
-        <f>IF(G44=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A44,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H44" s="14" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="45">
@@ -13573,9 +13590,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A45,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H45" s="14">
-        <f>IF(G45=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A45,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H45" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -13611,9 +13629,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A46,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H46" s="14">
-        <f>IF(G46=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A46,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H46" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -13649,9 +13668,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A47,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H47" s="14">
-        <f>IF(G47=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A47,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H47" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -13687,9 +13707,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A48,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H48" s="14">
-        <f>IF(G48=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A48,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H48" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -13725,9 +13746,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A49,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H49" s="14">
-        <f>IF(G49=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A49,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H49" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="50">
@@ -13763,9 +13785,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A50,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H50" s="14">
-        <f>IF(G50=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A50,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H50" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -13801,9 +13824,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A51,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H51" s="14">
-        <f>IF(G51=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A51,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H51" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="52">
@@ -13839,9 +13863,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A52,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H52" s="14">
-        <f>IF(G52=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A52,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H52" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="53">
@@ -13877,9 +13902,10 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A53,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H53" s="14">
-        <f>IF(G53=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A53,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H53" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="54">
@@ -13911,9 +13937,8 @@
         <f>COUNTIFS('Master Plan'!$D$2:$D$170,$A54,'Master Plan'!$K$2:$K$170,"&gt;0")</f>
         <v/>
       </c>
-      <c r="H54" s="14">
-        <f>IF(G54=0,"-",_xlfn.MINIFS('Master Plan'!$K$2:$K$170,'Master Plan'!$D$2:$D$170,$A54,'Master Plan'!$K$2:$K$170,"&gt;0"))</f>
-        <v/>
+      <c r="H54" s="14" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="56">

</xml_diff>